<commit_message>
Fix font color/size of September value cells in CENTRAL 50 and BENNETT
Brand value cells in the rebuilt September blocks had inconsistent font
(theme/size-12) vs the rest of the report. Normalize to match the report
convention: numbers in dark FF1F1F1F, dashes in grey FFA6A6A6, Calibri 10.5.
Headers, total rows and daily-total formatting left unchanged.
</commit_message>
<xml_diff>
--- a/MONTHLY SALES REPORT - ALL ZONES (PetPooja style) (1) (2).xlsx
+++ b/MONTHLY SALES REPORT - ALL ZONES (PetPooja style) (1) (2).xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[&gt;=10000000]&quot;₹&quot;##\,##\,##\,##0;[&gt;=100000]&quot;₹&quot;##\,##\,##0;&quot;₹&quot;#,##0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -161,6 +161,18 @@
       <charset val="1"/>
       <color theme="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <strike val="0"/>
+      <color rgb="FF1F1F1F"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <strike val="0"/>
+      <color rgb="FFA6A6A6"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
   <fills count="9">
@@ -363,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -480,6 +492,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -26137,22 +26179,22 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C360" s="24" t="n">
+      <c r="C360" s="42" t="n">
         <v>17549</v>
       </c>
-      <c r="D360" s="24" t="n">
+      <c r="D360" s="42" t="n">
         <v>9232</v>
       </c>
-      <c r="E360" s="28" t="n">
+      <c r="E360" s="42" t="n">
         <v>21114</v>
       </c>
-      <c r="F360" s="24" t="n">
+      <c r="F360" s="42" t="n">
         <v>7287</v>
       </c>
-      <c r="G360" s="24" t="n">
+      <c r="G360" s="42" t="n">
         <v>8898</v>
       </c>
-      <c r="H360" s="24" t="inlineStr">
+      <c r="H360" s="43" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -26172,22 +26214,22 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C361" s="25" t="n">
+      <c r="C361" s="44" t="n">
         <v>29793</v>
       </c>
-      <c r="D361" s="25" t="n">
+      <c r="D361" s="44" t="n">
         <v>18699</v>
       </c>
-      <c r="E361" s="29" t="n">
+      <c r="E361" s="44" t="n">
         <v>25299</v>
       </c>
-      <c r="F361" s="25" t="n">
+      <c r="F361" s="44" t="n">
         <v>8232</v>
       </c>
-      <c r="G361" s="25" t="n">
+      <c r="G361" s="44" t="n">
         <v>12509</v>
       </c>
-      <c r="H361" s="25" t="inlineStr">
+      <c r="H361" s="45" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -26207,22 +26249,22 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C362" s="25" t="n">
+      <c r="C362" s="44" t="n">
         <v>20814</v>
       </c>
-      <c r="D362" s="25" t="n">
+      <c r="D362" s="44" t="n">
         <v>20072</v>
       </c>
-      <c r="E362" s="29" t="n">
+      <c r="E362" s="44" t="n">
         <v>24729</v>
       </c>
-      <c r="F362" s="25" t="n">
+      <c r="F362" s="44" t="n">
         <v>18225</v>
       </c>
-      <c r="G362" s="25" t="n">
+      <c r="G362" s="44" t="n">
         <v>15119</v>
       </c>
-      <c r="H362" s="25" t="inlineStr">
+      <c r="H362" s="45" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -26242,22 +26284,22 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C363" s="25" t="n">
+      <c r="C363" s="44" t="n">
         <v>23498</v>
       </c>
-      <c r="D363" s="25" t="n">
+      <c r="D363" s="44" t="n">
         <v>14672</v>
       </c>
-      <c r="E363" s="29" t="n">
+      <c r="E363" s="44" t="n">
         <v>23398</v>
       </c>
-      <c r="F363" s="25" t="n">
+      <c r="F363" s="44" t="n">
         <v>10817</v>
       </c>
-      <c r="G363" s="25" t="n">
+      <c r="G363" s="44" t="n">
         <v>14340</v>
       </c>
-      <c r="H363" s="25" t="inlineStr">
+      <c r="H363" s="45" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -26277,22 +26319,22 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C364" s="25" t="n">
+      <c r="C364" s="44" t="n">
         <v>60927</v>
       </c>
-      <c r="D364" s="25" t="n">
+      <c r="D364" s="44" t="n">
         <v>33009</v>
       </c>
-      <c r="E364" s="29" t="n">
+      <c r="E364" s="44" t="n">
         <v>71074</v>
       </c>
-      <c r="F364" s="25" t="n">
+      <c r="F364" s="44" t="n">
         <v>34184</v>
       </c>
-      <c r="G364" s="25" t="n">
+      <c r="G364" s="44" t="n">
         <v>34250</v>
       </c>
-      <c r="H364" s="25" t="n">
+      <c r="H364" s="44" t="n">
         <v>4781</v>
       </c>
       <c r="I364" s="6" t="n">
@@ -26310,22 +26352,22 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C365" s="25" t="n">
+      <c r="C365" s="44" t="n">
         <v>74767</v>
       </c>
-      <c r="D365" s="25" t="n">
+      <c r="D365" s="44" t="n">
         <v>41148</v>
       </c>
-      <c r="E365" s="29" t="n">
+      <c r="E365" s="44" t="n">
         <v>60464</v>
       </c>
-      <c r="F365" s="25" t="n">
+      <c r="F365" s="44" t="n">
         <v>32988</v>
       </c>
-      <c r="G365" s="25" t="n">
+      <c r="G365" s="44" t="n">
         <v>43877</v>
       </c>
-      <c r="H365" s="25" t="n">
+      <c r="H365" s="44" t="n">
         <v>7087</v>
       </c>
       <c r="I365" s="6" t="n">
@@ -26343,22 +26385,22 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C366" s="25" t="n">
+      <c r="C366" s="44" t="n">
         <v>30850</v>
       </c>
-      <c r="D366" s="25" t="n">
+      <c r="D366" s="44" t="n">
         <v>10691</v>
       </c>
-      <c r="E366" s="29" t="n">
+      <c r="E366" s="44" t="n">
         <v>26623</v>
       </c>
-      <c r="F366" s="25" t="n">
+      <c r="F366" s="44" t="n">
         <v>10929</v>
       </c>
-      <c r="G366" s="25" t="n">
+      <c r="G366" s="44" t="n">
         <v>17098</v>
       </c>
-      <c r="H366" s="25" t="n">
+      <c r="H366" s="44" t="n">
         <v>1332</v>
       </c>
       <c r="I366" s="6" t="n">
@@ -26376,22 +26418,22 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C367" s="25" t="n">
+      <c r="C367" s="44" t="n">
         <v>28191</v>
       </c>
-      <c r="D367" s="25" t="n">
+      <c r="D367" s="44" t="n">
         <v>10921</v>
       </c>
-      <c r="E367" s="29" t="n">
+      <c r="E367" s="44" t="n">
         <v>23487</v>
       </c>
-      <c r="F367" s="25" t="n">
+      <c r="F367" s="44" t="n">
         <v>10178</v>
       </c>
-      <c r="G367" s="25" t="n">
+      <c r="G367" s="44" t="n">
         <v>15046</v>
       </c>
-      <c r="H367" s="25" t="n">
+      <c r="H367" s="44" t="n">
         <v>2406</v>
       </c>
       <c r="I367" s="6" t="n">
@@ -26409,22 +26451,22 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C368" s="25" t="n">
+      <c r="C368" s="44" t="n">
         <v>28175</v>
       </c>
-      <c r="D368" s="25" t="n">
+      <c r="D368" s="44" t="n">
         <v>14003</v>
       </c>
-      <c r="E368" s="29" t="n">
+      <c r="E368" s="44" t="n">
         <v>23356</v>
       </c>
-      <c r="F368" s="25" t="n">
+      <c r="F368" s="44" t="n">
         <v>12464</v>
       </c>
-      <c r="G368" s="25" t="n">
+      <c r="G368" s="44" t="n">
         <v>11216</v>
       </c>
-      <c r="H368" s="25" t="n">
+      <c r="H368" s="44" t="n">
         <v>2844</v>
       </c>
       <c r="I368" s="6" t="n">
@@ -26442,22 +26484,22 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C369" s="25" t="n">
+      <c r="C369" s="44" t="n">
         <v>24677</v>
       </c>
-      <c r="D369" s="25" t="n">
+      <c r="D369" s="44" t="n">
         <v>17230</v>
       </c>
-      <c r="E369" s="29" t="n">
+      <c r="E369" s="44" t="n">
         <v>25694</v>
       </c>
-      <c r="F369" s="30" t="n">
+      <c r="F369" s="44" t="n">
         <v>9989</v>
       </c>
-      <c r="G369" s="29" t="n">
+      <c r="G369" s="44" t="n">
         <v>15095</v>
       </c>
-      <c r="H369" s="29" t="n">
+      <c r="H369" s="44" t="n">
         <v>1561</v>
       </c>
       <c r="I369" s="6" t="n">
@@ -26475,22 +26517,22 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C370" s="26" t="n">
+      <c r="C370" s="46" t="n">
         <v>35697</v>
       </c>
-      <c r="D370" s="25" t="n">
+      <c r="D370" s="44" t="n">
         <v>22769</v>
       </c>
-      <c r="E370" s="29" t="n">
+      <c r="E370" s="44" t="n">
         <v>37384</v>
       </c>
-      <c r="F370" s="25" t="n">
+      <c r="F370" s="44" t="n">
         <v>18637</v>
       </c>
-      <c r="G370" s="25" t="n">
+      <c r="G370" s="44" t="n">
         <v>22327</v>
       </c>
-      <c r="H370" s="25" t="n">
+      <c r="H370" s="44" t="n">
         <v>5319</v>
       </c>
       <c r="I370" s="6" t="n">
@@ -26508,22 +26550,22 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C371" s="25" t="n">
+      <c r="C371" s="44" t="n">
         <v>74337</v>
       </c>
-      <c r="D371" s="25" t="n">
+      <c r="D371" s="44" t="n">
         <v>41066</v>
       </c>
-      <c r="E371" s="29" t="n">
+      <c r="E371" s="44" t="n">
         <v>73148</v>
       </c>
-      <c r="F371" s="25" t="n">
+      <c r="F371" s="44" t="n">
         <v>24739</v>
       </c>
-      <c r="G371" s="25" t="n">
+      <c r="G371" s="44" t="n">
         <v>36125</v>
       </c>
-      <c r="H371" s="25" t="n">
+      <c r="H371" s="44" t="n">
         <v>10736</v>
       </c>
       <c r="I371" s="6" t="n">
@@ -26541,22 +26583,22 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C372" s="25" t="n">
+      <c r="C372" s="44" t="n">
         <v>66843</v>
       </c>
-      <c r="D372" s="25" t="n">
+      <c r="D372" s="44" t="n">
         <v>42637</v>
       </c>
-      <c r="E372" s="29" t="n">
+      <c r="E372" s="44" t="n">
         <v>62011</v>
       </c>
-      <c r="F372" s="25" t="n">
+      <c r="F372" s="44" t="n">
         <v>28271</v>
       </c>
-      <c r="G372" s="25" t="n">
+      <c r="G372" s="44" t="n">
         <v>47519</v>
       </c>
-      <c r="H372" s="25" t="n">
+      <c r="H372" s="44" t="n">
         <v>7307</v>
       </c>
       <c r="I372" s="6" t="n">
@@ -26574,22 +26616,22 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C373" s="25" t="n">
+      <c r="C373" s="44" t="n">
         <v>26863</v>
       </c>
-      <c r="D373" s="25" t="n">
+      <c r="D373" s="44" t="n">
         <v>15761</v>
       </c>
-      <c r="E373" s="29" t="n">
+      <c r="E373" s="44" t="n">
         <v>20455</v>
       </c>
-      <c r="F373" s="25" t="n">
+      <c r="F373" s="44" t="n">
         <v>10358</v>
       </c>
-      <c r="G373" s="25" t="n">
+      <c r="G373" s="44" t="n">
         <v>16891</v>
       </c>
-      <c r="H373" s="25" t="n">
+      <c r="H373" s="44" t="n">
         <v>2008</v>
       </c>
       <c r="I373" s="6" t="n">
@@ -26607,22 +26649,22 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C374" s="25" t="n">
+      <c r="C374" s="44" t="n">
         <v>26429</v>
       </c>
-      <c r="D374" s="25" t="n">
+      <c r="D374" s="44" t="n">
         <v>13098</v>
       </c>
-      <c r="E374" s="29" t="n">
+      <c r="E374" s="44" t="n">
         <v>19784</v>
       </c>
-      <c r="F374" s="25" t="n">
+      <c r="F374" s="44" t="n">
         <v>9022</v>
       </c>
-      <c r="G374" s="25" t="n">
+      <c r="G374" s="44" t="n">
         <v>15609</v>
       </c>
-      <c r="H374" s="25" t="n">
+      <c r="H374" s="44" t="n">
         <v>1392</v>
       </c>
       <c r="I374" s="6" t="n">
@@ -26640,22 +26682,22 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C375" s="25" t="n">
+      <c r="C375" s="44" t="n">
         <v>15839</v>
       </c>
-      <c r="D375" s="25" t="n">
+      <c r="D375" s="44" t="n">
         <v>16419</v>
       </c>
-      <c r="E375" s="29" t="n">
+      <c r="E375" s="44" t="n">
         <v>26386</v>
       </c>
-      <c r="F375" s="25" t="n">
+      <c r="F375" s="44" t="n">
         <v>7401</v>
       </c>
-      <c r="G375" s="25" t="n">
+      <c r="G375" s="44" t="n">
         <v>13813</v>
       </c>
-      <c r="H375" s="25" t="n">
+      <c r="H375" s="44" t="n">
         <v>1872</v>
       </c>
       <c r="I375" s="6" t="n">
@@ -26673,22 +26715,22 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C376" s="25" t="n">
+      <c r="C376" s="44" t="n">
         <v>31967</v>
       </c>
-      <c r="D376" s="25" t="n">
+      <c r="D376" s="44" t="n">
         <v>18297</v>
       </c>
-      <c r="E376" s="29" t="n">
+      <c r="E376" s="44" t="n">
         <v>29457</v>
       </c>
-      <c r="F376" s="25" t="n">
+      <c r="F376" s="44" t="n">
         <v>9847</v>
       </c>
-      <c r="G376" s="25" t="n">
+      <c r="G376" s="44" t="n">
         <v>19442</v>
       </c>
-      <c r="H376" s="25" t="n">
+      <c r="H376" s="44" t="n">
         <v>4125</v>
       </c>
       <c r="I376" s="6" t="n">
@@ -26706,22 +26748,22 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C377" s="25" t="n">
+      <c r="C377" s="44" t="n">
         <v>33719</v>
       </c>
-      <c r="D377" s="25" t="n">
+      <c r="D377" s="44" t="n">
         <v>21398</v>
       </c>
-      <c r="E377" s="29" t="n">
+      <c r="E377" s="44" t="n">
         <v>28176</v>
       </c>
-      <c r="F377" s="25" t="n">
+      <c r="F377" s="44" t="n">
         <v>21331</v>
       </c>
-      <c r="G377" s="25" t="n">
+      <c r="G377" s="44" t="n">
         <v>19409</v>
       </c>
-      <c r="H377" s="25" t="n">
+      <c r="H377" s="44" t="n">
         <v>4176</v>
       </c>
       <c r="I377" s="6" t="n">
@@ -26739,22 +26781,22 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C378" s="25" t="n">
+      <c r="C378" s="44" t="n">
         <v>59554</v>
       </c>
-      <c r="D378" s="25" t="n">
+      <c r="D378" s="44" t="n">
         <v>40918</v>
       </c>
-      <c r="E378" s="29" t="n">
+      <c r="E378" s="44" t="n">
         <v>62027</v>
       </c>
-      <c r="F378" s="25" t="n">
+      <c r="F378" s="44" t="n">
         <v>30348</v>
       </c>
-      <c r="G378" s="25" t="n">
+      <c r="G378" s="44" t="n">
         <v>37412</v>
       </c>
-      <c r="H378" s="25" t="n">
+      <c r="H378" s="44" t="n">
         <v>7238</v>
       </c>
       <c r="I378" s="6" t="n">
@@ -26772,22 +26814,22 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C379" s="25" t="n">
+      <c r="C379" s="44" t="n">
         <v>55295</v>
       </c>
-      <c r="D379" s="25" t="n">
+      <c r="D379" s="44" t="n">
         <v>47545</v>
       </c>
-      <c r="E379" s="29" t="n">
+      <c r="E379" s="44" t="n">
         <v>61752</v>
       </c>
-      <c r="F379" s="25" t="n">
+      <c r="F379" s="44" t="n">
         <v>27138</v>
       </c>
-      <c r="G379" s="29" t="n">
+      <c r="G379" s="44" t="n">
         <v>38573</v>
       </c>
-      <c r="H379" s="29" t="n">
+      <c r="H379" s="44" t="n">
         <v>10829</v>
       </c>
       <c r="I379" s="6" t="n">
@@ -26805,22 +26847,22 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C380" s="25" t="n">
+      <c r="C380" s="44" t="n">
         <v>19354</v>
       </c>
-      <c r="D380" s="25" t="n">
+      <c r="D380" s="44" t="n">
         <v>15579</v>
       </c>
-      <c r="E380" s="29" t="n">
+      <c r="E380" s="44" t="n">
         <v>23158</v>
       </c>
-      <c r="F380" s="25" t="n">
+      <c r="F380" s="44" t="n">
         <v>9861</v>
       </c>
-      <c r="G380" s="25" t="n">
+      <c r="G380" s="44" t="n">
         <v>13754</v>
       </c>
-      <c r="H380" s="25" t="n">
+      <c r="H380" s="44" t="n">
         <v>2784</v>
       </c>
       <c r="I380" s="6" t="n">
@@ -26838,22 +26880,22 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C381" s="27" t="n">
+      <c r="C381" s="47" t="n">
         <v>16269</v>
       </c>
-      <c r="D381" s="25" t="n">
+      <c r="D381" s="44" t="n">
         <v>13343</v>
       </c>
-      <c r="E381" s="29" t="n">
+      <c r="E381" s="44" t="n">
         <v>21899</v>
       </c>
-      <c r="F381" s="25" t="n">
+      <c r="F381" s="44" t="n">
         <v>11271</v>
       </c>
-      <c r="G381" s="25" t="n">
+      <c r="G381" s="44" t="n">
         <v>14160</v>
       </c>
-      <c r="H381" s="25" t="n">
+      <c r="H381" s="44" t="n">
         <v>1681</v>
       </c>
       <c r="I381" s="6" t="n">
@@ -26871,22 +26913,22 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C382" s="27" t="n">
+      <c r="C382" s="47" t="n">
         <v>24649</v>
       </c>
-      <c r="D382" s="25" t="n">
+      <c r="D382" s="44" t="n">
         <v>14269</v>
       </c>
-      <c r="E382" s="29" t="n">
+      <c r="E382" s="44" t="n">
         <v>22995</v>
       </c>
-      <c r="F382" s="25" t="n">
+      <c r="F382" s="44" t="n">
         <v>11312</v>
       </c>
-      <c r="G382" s="25" t="n">
+      <c r="G382" s="44" t="n">
         <v>13856</v>
       </c>
-      <c r="H382" s="25" t="n">
+      <c r="H382" s="44" t="n">
         <v>3724</v>
       </c>
       <c r="I382" s="6" t="n">
@@ -26904,22 +26946,22 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C383" s="27" t="n">
+      <c r="C383" s="47" t="n">
         <v>28689</v>
       </c>
-      <c r="D383" s="25" t="n">
+      <c r="D383" s="44" t="n">
         <v>14520</v>
       </c>
-      <c r="E383" s="29" t="n">
+      <c r="E383" s="44" t="n">
         <v>30752</v>
       </c>
-      <c r="F383" s="25" t="n">
+      <c r="F383" s="44" t="n">
         <v>14560</v>
       </c>
-      <c r="G383" s="25" t="n">
+      <c r="G383" s="44" t="n">
         <v>23531</v>
       </c>
-      <c r="H383" s="25" t="n">
+      <c r="H383" s="44" t="n">
         <v>2973</v>
       </c>
       <c r="I383" s="6" t="n">
@@ -26937,22 +26979,22 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C384" s="25" t="n">
+      <c r="C384" s="44" t="n">
         <v>37148</v>
       </c>
-      <c r="D384" s="25" t="n">
+      <c r="D384" s="44" t="n">
         <v>25116</v>
       </c>
-      <c r="E384" s="29" t="n">
+      <c r="E384" s="44" t="n">
         <v>53284</v>
       </c>
-      <c r="F384" s="25" t="n">
+      <c r="F384" s="44" t="n">
         <v>19756</v>
       </c>
-      <c r="G384" s="25" t="n">
+      <c r="G384" s="44" t="n">
         <v>26399</v>
       </c>
-      <c r="H384" s="25" t="n">
+      <c r="H384" s="44" t="n">
         <v>4942</v>
       </c>
       <c r="I384" s="6" t="n">
@@ -26970,22 +27012,22 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C385" s="25" t="n">
+      <c r="C385" s="44" t="n">
         <v>50635</v>
       </c>
-      <c r="D385" s="25" t="n">
+      <c r="D385" s="44" t="n">
         <v>24420</v>
       </c>
-      <c r="E385" s="29" t="n">
+      <c r="E385" s="44" t="n">
         <v>55676</v>
       </c>
-      <c r="F385" s="25" t="n">
+      <c r="F385" s="44" t="n">
         <v>21682</v>
       </c>
-      <c r="G385" s="25" t="n">
+      <c r="G385" s="44" t="n">
         <v>30988</v>
       </c>
-      <c r="H385" s="25" t="n">
+      <c r="H385" s="44" t="n">
         <v>8639</v>
       </c>
       <c r="I385" s="6" t="n">
@@ -27003,22 +27045,22 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C386" s="25" t="n">
+      <c r="C386" s="44" t="n">
         <v>78437</v>
       </c>
-      <c r="D386" s="25" t="n">
+      <c r="D386" s="44" t="n">
         <v>40661</v>
       </c>
-      <c r="E386" s="29" t="n">
+      <c r="E386" s="44" t="n">
         <v>70042</v>
       </c>
-      <c r="F386" s="25" t="n">
+      <c r="F386" s="44" t="n">
         <v>53655</v>
       </c>
-      <c r="G386" s="29" t="n">
+      <c r="G386" s="44" t="n">
         <v>63686</v>
       </c>
-      <c r="H386" s="29" t="n">
+      <c r="H386" s="44" t="n">
         <v>16489</v>
       </c>
       <c r="I386" s="6" t="n">
@@ -27036,22 +27078,22 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C387" s="25" t="n">
+      <c r="C387" s="44" t="n">
         <v>21760</v>
       </c>
-      <c r="D387" s="25" t="n">
+      <c r="D387" s="44" t="n">
         <v>13016</v>
       </c>
-      <c r="E387" s="29" t="n">
+      <c r="E387" s="44" t="n">
         <v>29560</v>
       </c>
-      <c r="F387" s="25" t="n">
+      <c r="F387" s="44" t="n">
         <v>13993</v>
       </c>
-      <c r="G387" s="25" t="n">
+      <c r="G387" s="44" t="n">
         <v>18200</v>
       </c>
-      <c r="H387" s="25" t="n">
+      <c r="H387" s="44" t="n">
         <v>5039</v>
       </c>
       <c r="I387" s="22" t="n">
@@ -27069,22 +27111,22 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C388" s="25" t="n">
+      <c r="C388" s="44" t="n">
         <v>26727</v>
       </c>
-      <c r="D388" s="25" t="n">
+      <c r="D388" s="44" t="n">
         <v>15000</v>
       </c>
-      <c r="E388" s="25" t="n">
+      <c r="E388" s="44" t="n">
         <v>23840</v>
       </c>
-      <c r="F388" s="25" t="n">
+      <c r="F388" s="44" t="n">
         <v>13590</v>
       </c>
-      <c r="G388" s="25" t="n">
+      <c r="G388" s="44" t="n">
         <v>12924</v>
       </c>
-      <c r="H388" s="25" t="n">
+      <c r="H388" s="44" t="n">
         <v>3798</v>
       </c>
       <c r="I388" s="22" t="n">
@@ -27102,22 +27144,22 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C389" s="25" t="n">
+      <c r="C389" s="44" t="n">
         <v>19305</v>
       </c>
-      <c r="D389" s="25" t="n">
+      <c r="D389" s="44" t="n">
         <v>15685</v>
       </c>
-      <c r="E389" s="29" t="n">
+      <c r="E389" s="44" t="n">
         <v>29718</v>
       </c>
-      <c r="F389" s="25" t="n">
+      <c r="F389" s="44" t="n">
         <v>13828</v>
       </c>
-      <c r="G389" s="25" t="n">
+      <c r="G389" s="44" t="n">
         <v>9180</v>
       </c>
-      <c r="H389" s="25" t="n">
+      <c r="H389" s="44" t="n">
         <v>5219</v>
       </c>
       <c r="I389" s="22" t="n">
@@ -31867,7 +31909,7 @@
       <c r="J90" s="10" t="n">
         <v>4234</v>
       </c>
-      <c r="K90" s="10" t="inlineStr">
+      <c r="K90" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -31914,7 +31956,7 @@
       <c r="J91" s="15" t="n">
         <v>3967</v>
       </c>
-      <c r="K91" s="15" t="inlineStr">
+      <c r="K91" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -31961,7 +32003,7 @@
       <c r="J92" s="15" t="n">
         <v>5068</v>
       </c>
-      <c r="K92" s="15" t="inlineStr">
+      <c r="K92" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32008,7 +32050,7 @@
       <c r="J93" s="15" t="n">
         <v>5494</v>
       </c>
-      <c r="K93" s="15" t="inlineStr">
+      <c r="K93" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32055,7 +32097,7 @@
       <c r="J94" s="15" t="n">
         <v>8613</v>
       </c>
-      <c r="K94" s="15" t="inlineStr">
+      <c r="K94" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32102,7 +32144,7 @@
       <c r="J95" s="15" t="n">
         <v>2376</v>
       </c>
-      <c r="K95" s="15" t="inlineStr">
+      <c r="K95" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32149,7 +32191,7 @@
       <c r="J96" s="10" t="n">
         <v>3257</v>
       </c>
-      <c r="K96" s="10" t="inlineStr">
+      <c r="K96" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32196,7 +32238,7 @@
       <c r="J97" s="10" t="n">
         <v>2951</v>
       </c>
-      <c r="K97" s="10" t="inlineStr">
+      <c r="K97" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32243,7 +32285,7 @@
       <c r="J98" s="15" t="n">
         <v>2483</v>
       </c>
-      <c r="K98" s="15" t="inlineStr">
+      <c r="K98" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32290,7 +32332,7 @@
       <c r="J99" s="15" t="n">
         <v>4226</v>
       </c>
-      <c r="K99" s="15" t="inlineStr">
+      <c r="K99" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32337,7 +32379,7 @@
       <c r="J100" s="15" t="n">
         <v>6556</v>
       </c>
-      <c r="K100" s="15" t="inlineStr">
+      <c r="K100" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32375,7 +32417,7 @@
       <c r="G101" s="15" t="n">
         <v>66113</v>
       </c>
-      <c r="H101" s="9" t="n">
+      <c r="H101" s="50" t="n">
         <v>4575</v>
       </c>
       <c r="I101" s="15" t="n">
@@ -32384,7 +32426,7 @@
       <c r="J101" s="15" t="n">
         <v>7387</v>
       </c>
-      <c r="K101" s="15" t="inlineStr">
+      <c r="K101" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32422,7 +32464,7 @@
       <c r="G102" s="15" t="n">
         <v>82534</v>
       </c>
-      <c r="H102" s="9" t="n">
+      <c r="H102" s="50" t="n">
         <v>3568</v>
       </c>
       <c r="I102" s="15" t="n">
@@ -32431,7 +32473,7 @@
       <c r="J102" s="15" t="n">
         <v>10087</v>
       </c>
-      <c r="K102" s="15" t="inlineStr">
+      <c r="K102" s="49" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32469,7 +32511,7 @@
       <c r="G103" s="10" t="n">
         <v>55960</v>
       </c>
-      <c r="H103" s="5" t="n">
+      <c r="H103" s="51" t="n">
         <v>1569</v>
       </c>
       <c r="I103" s="10" t="n">
@@ -32478,7 +32520,7 @@
       <c r="J103" s="10" t="n">
         <v>1661</v>
       </c>
-      <c r="K103" s="10" t="inlineStr">
+      <c r="K103" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32516,7 +32558,7 @@
       <c r="G104" s="10" t="n">
         <v>70457</v>
       </c>
-      <c r="H104" s="5" t="n">
+      <c r="H104" s="51" t="n">
         <v>3888</v>
       </c>
       <c r="I104" s="10" t="n">
@@ -32525,7 +32567,7 @@
       <c r="J104" s="10" t="n">
         <v>12805</v>
       </c>
-      <c r="K104" s="10" t="inlineStr">
+      <c r="K104" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -32548,7 +32590,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C105" s="9" t="n">
+      <c r="C105" s="50" t="n">
         <v>25355</v>
       </c>
       <c r="D105" s="15" t="n">
@@ -32560,7 +32602,7 @@
       <c r="F105" s="15" t="n">
         <v>10561</v>
       </c>
-      <c r="G105" s="9" t="n">
+      <c r="G105" s="50" t="n">
         <v>72137</v>
       </c>
       <c r="H105" s="15" t="n">
@@ -32569,10 +32611,10 @@
       <c r="I105" s="15" t="n">
         <v>8082</v>
       </c>
-      <c r="J105" s="9" t="n">
+      <c r="J105" s="50" t="n">
         <v>11547</v>
       </c>
-      <c r="K105" s="9" t="n">
+      <c r="K105" s="50" t="n">
         <v>6580</v>
       </c>
       <c r="L105" s="15" t="n">
@@ -32593,7 +32635,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C106" s="9" t="n">
+      <c r="C106" s="50" t="n">
         <v>28290</v>
       </c>
       <c r="D106" s="15" t="n">
@@ -32605,7 +32647,7 @@
       <c r="F106" s="15" t="n">
         <v>8427</v>
       </c>
-      <c r="G106" s="9" t="n">
+      <c r="G106" s="50" t="n">
         <v>94544</v>
       </c>
       <c r="H106" s="15" t="n">
@@ -32614,10 +32656,10 @@
       <c r="I106" s="15" t="n">
         <v>9321</v>
       </c>
-      <c r="J106" s="9" t="n">
+      <c r="J106" s="50" t="n">
         <v>14156</v>
       </c>
-      <c r="K106" s="9" t="n">
+      <c r="K106" s="50" t="n">
         <v>6422</v>
       </c>
       <c r="L106" s="15" t="n">
@@ -32638,7 +32680,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C107" s="9" t="n">
+      <c r="C107" s="50" t="n">
         <v>25881</v>
       </c>
       <c r="D107" s="15" t="n">
@@ -32650,7 +32692,7 @@
       <c r="F107" s="15" t="n">
         <v>9527</v>
       </c>
-      <c r="G107" s="9" t="n">
+      <c r="G107" s="50" t="n">
         <v>91515</v>
       </c>
       <c r="H107" s="15" t="n">
@@ -32659,10 +32701,10 @@
       <c r="I107" s="15" t="n">
         <v>7328</v>
       </c>
-      <c r="J107" s="9" t="n">
+      <c r="J107" s="50" t="n">
         <v>14456</v>
       </c>
-      <c r="K107" s="9" t="n">
+      <c r="K107" s="50" t="n">
         <v>9014</v>
       </c>
       <c r="L107" s="15" t="n">
@@ -32734,7 +32776,6 @@
       </c>
       <c r="M109" s="41" t="n"/>
     </row>
-    <row r="110"/>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
         <is>
@@ -32805,8 +32846,8 @@
   <mergeCells count="13">
     <mergeCell ref="A76:M76"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="L38:M38"/>
     <mergeCell ref="A74:J74"/>
-    <mergeCell ref="L38:M38"/>
     <mergeCell ref="L109:M109"/>
     <mergeCell ref="A40:M40"/>
     <mergeCell ref="A4:M4"/>

</xml_diff>

<commit_message>
Add new zone sheet: CAPITAL ATHENA SECTOR-1 (September 2026)
New zone with brands MOMO BOX, THE COFFEE VAULT, THE CHATPATA AFFAIR.
September daily data (18-30 Sep), same PetPooja-style formatting as other
zones: blue header, weekend shading, cream total row, INR number format,
grey dashes for no-sale days. Zone total Rs.2,55,436.03.
</commit_message>
<xml_diff>
--- a/MONTHLY SALES REPORT - ALL ZONES (PetPooja style) (1) (2).xlsx
+++ b/MONTHLY SALES REPORT - ALL ZONES (PetPooja style) (1) (2).xlsx
@@ -10,6 +10,7 @@
     <sheet name="CENTRAL 50" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="BENNETT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="DISTRICT 9" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CAPITAL ATHENA SECTOR-1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[&gt;=10000000]&quot;₹&quot;##\,##\,##\,##0;[&gt;=100000]&quot;₹&quot;##\,##\,##0;&quot;₹&quot;#,##0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -174,6 +175,11 @@
       <color rgb="FFA6A6A6"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF666666"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -220,7 +226,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -371,11 +377,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF2E5A87"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -521,6 +569,69 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -34292,4 +34403,952 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" style="32" min="1" max="1"/>
+    <col width="12" customWidth="1" style="32" min="2" max="2"/>
+    <col width="15" customWidth="1" style="32" min="3" max="3"/>
+    <col width="16" customWidth="1" style="32" min="4" max="4"/>
+    <col width="18" customWidth="1" style="32" min="5" max="5"/>
+    <col width="16" customWidth="1" style="32" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26.1" customHeight="1" s="32">
+      <c r="A1" s="52" t="inlineStr">
+        <is>
+          <t>CAPITAL ATHENA SECTOR-1  —  MONTHLY DAILY-BRAND SALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.95" customHeight="1" s="32">
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Day-wise net sales by brand  •  September 2026  •  Amounts in ₹ (INR)  •  weekend rows shaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="21.95" customHeight="1" s="32">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>September 2026. -  ZONE CAPITAL ATHENA SECTOR - 1</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="n"/>
+      <c r="C4" s="40" t="n"/>
+      <c r="D4" s="40" t="n"/>
+      <c r="E4" s="40" t="n"/>
+      <c r="F4" s="41" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="32">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>MOMO BOX</t>
+        </is>
+      </c>
+      <c r="D5" s="56" t="inlineStr">
+        <is>
+          <t>THE COFFEE VAULT</t>
+        </is>
+      </c>
+      <c r="E5" s="56" t="inlineStr">
+        <is>
+          <t>THE CHATPATA AFFAIR</t>
+        </is>
+      </c>
+      <c r="F5" s="55" t="inlineStr">
+        <is>
+          <t>TOTAL ZONE SALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.1" customHeight="1" s="32">
+      <c r="A6" s="57" t="inlineStr">
+        <is>
+          <t>01 Sep</t>
+        </is>
+      </c>
+      <c r="B6" s="58" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C6" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D6" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E6" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F6" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="17.1" customHeight="1" s="32">
+      <c r="A7" s="57" t="inlineStr">
+        <is>
+          <t>02 Sep</t>
+        </is>
+      </c>
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C7" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D7" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E7" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F7" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="17.1" customHeight="1" s="32">
+      <c r="A8" s="57" t="inlineStr">
+        <is>
+          <t>03 Sep</t>
+        </is>
+      </c>
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D8" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E8" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F8" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="17.1" customHeight="1" s="32">
+      <c r="A9" s="57" t="inlineStr">
+        <is>
+          <t>04 Sep</t>
+        </is>
+      </c>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C9" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D9" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E9" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F9" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="17.1" customHeight="1" s="32">
+      <c r="A10" s="61" t="inlineStr">
+        <is>
+          <t>05 Sep</t>
+        </is>
+      </c>
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C10" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D10" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E10" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F10" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="17.1" customHeight="1" s="32">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>06 Sep</t>
+        </is>
+      </c>
+      <c r="B11" s="62" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F11" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="17.1" customHeight="1" s="32">
+      <c r="A12" s="57" t="inlineStr">
+        <is>
+          <t>07 Sep</t>
+        </is>
+      </c>
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F12" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="17.1" customHeight="1" s="32">
+      <c r="A13" s="57" t="inlineStr">
+        <is>
+          <t>08 Sep</t>
+        </is>
+      </c>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E13" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F13" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="17.1" customHeight="1" s="32">
+      <c r="A14" s="57" t="inlineStr">
+        <is>
+          <t>09 Sep</t>
+        </is>
+      </c>
+      <c r="B14" s="58" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C14" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E14" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F14" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="17.1" customHeight="1" s="32">
+      <c r="A15" s="57" t="inlineStr">
+        <is>
+          <t>10 Sep</t>
+        </is>
+      </c>
+      <c r="B15" s="58" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C15" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D15" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E15" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F15" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="17.1" customHeight="1" s="32">
+      <c r="A16" s="57" t="inlineStr">
+        <is>
+          <t>11 Sep</t>
+        </is>
+      </c>
+      <c r="B16" s="58" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="17.1" customHeight="1" s="32">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>12 Sep</t>
+        </is>
+      </c>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="17.1" customHeight="1" s="32">
+      <c r="A18" s="61" t="inlineStr">
+        <is>
+          <t>13 Sep</t>
+        </is>
+      </c>
+      <c r="B18" s="62" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C18" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D18" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E18" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F18" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="17.1" customHeight="1" s="32">
+      <c r="A19" s="57" t="inlineStr">
+        <is>
+          <t>14 Sep</t>
+        </is>
+      </c>
+      <c r="B19" s="58" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F19" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="17.1" customHeight="1" s="32">
+      <c r="A20" s="57" t="inlineStr">
+        <is>
+          <t>15 Sep</t>
+        </is>
+      </c>
+      <c r="B20" s="58" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E20" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F20" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="17.1" customHeight="1" s="32">
+      <c r="A21" s="57" t="inlineStr">
+        <is>
+          <t>16 Sep</t>
+        </is>
+      </c>
+      <c r="B21" s="58" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D21" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E21" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F21" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="17.1" customHeight="1" s="32">
+      <c r="A22" s="57" t="inlineStr">
+        <is>
+          <t>17 Sep</t>
+        </is>
+      </c>
+      <c r="B22" s="58" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D22" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E22" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F22" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="17.1" customHeight="1" s="32">
+      <c r="A23" s="57" t="inlineStr">
+        <is>
+          <t>18 Sep</t>
+        </is>
+      </c>
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D23" s="71" t="n">
+        <v>2728</v>
+      </c>
+      <c r="E23" s="59" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F23" s="60" t="n">
+        <v>2728</v>
+      </c>
+    </row>
+    <row r="24" ht="17.1" customHeight="1" s="32">
+      <c r="A24" s="61" t="inlineStr">
+        <is>
+          <t>19 Sep</t>
+        </is>
+      </c>
+      <c r="B24" s="62" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C24" s="72" t="n">
+        <v>11186</v>
+      </c>
+      <c r="D24" s="72" t="n">
+        <v>10830</v>
+      </c>
+      <c r="E24" s="63" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F24" s="60" t="n">
+        <v>22016</v>
+      </c>
+    </row>
+    <row r="25" ht="17.1" customHeight="1" s="32">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>20 Sep</t>
+        </is>
+      </c>
+      <c r="B25" s="62" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C25" s="72" t="n">
+        <v>12395</v>
+      </c>
+      <c r="D25" s="72" t="n">
+        <v>9202</v>
+      </c>
+      <c r="E25" s="72" t="n">
+        <v>175</v>
+      </c>
+      <c r="F25" s="60" t="n">
+        <v>21772</v>
+      </c>
+    </row>
+    <row r="26" ht="17.1" customHeight="1" s="32">
+      <c r="A26" s="57" t="inlineStr">
+        <is>
+          <t>21 Sep</t>
+        </is>
+      </c>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C26" s="71" t="n">
+        <v>6265</v>
+      </c>
+      <c r="D26" s="71" t="n">
+        <v>5245</v>
+      </c>
+      <c r="E26" s="71" t="n">
+        <v>3780</v>
+      </c>
+      <c r="F26" s="60" t="n">
+        <v>15290</v>
+      </c>
+    </row>
+    <row r="27" ht="17.1" customHeight="1" s="32">
+      <c r="A27" s="57" t="inlineStr">
+        <is>
+          <t>22 Sep</t>
+        </is>
+      </c>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="n">
+        <v>8001</v>
+      </c>
+      <c r="D27" s="71" t="n">
+        <v>4264</v>
+      </c>
+      <c r="E27" s="71" t="n">
+        <v>6325</v>
+      </c>
+      <c r="F27" s="60" t="n">
+        <v>18590</v>
+      </c>
+    </row>
+    <row r="28" ht="17.1" customHeight="1" s="32">
+      <c r="A28" s="57" t="inlineStr">
+        <is>
+          <t>23 Sep</t>
+        </is>
+      </c>
+      <c r="B28" s="58" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="n">
+        <v>7301</v>
+      </c>
+      <c r="D28" s="71" t="n">
+        <v>3679</v>
+      </c>
+      <c r="E28" s="71" t="n">
+        <v>4928.18</v>
+      </c>
+      <c r="F28" s="60" t="n">
+        <v>15908.18</v>
+      </c>
+    </row>
+    <row r="29" ht="17.1" customHeight="1" s="32">
+      <c r="A29" s="57" t="inlineStr">
+        <is>
+          <t>24 Sep</t>
+        </is>
+      </c>
+      <c r="B29" s="58" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="n">
+        <v>6151</v>
+      </c>
+      <c r="D29" s="71" t="n">
+        <v>5888</v>
+      </c>
+      <c r="E29" s="71" t="n">
+        <v>4848.9</v>
+      </c>
+      <c r="F29" s="60" t="n">
+        <v>16887.9</v>
+      </c>
+    </row>
+    <row r="30" ht="17.1" customHeight="1" s="32">
+      <c r="A30" s="57" t="inlineStr">
+        <is>
+          <t>25 Sep</t>
+        </is>
+      </c>
+      <c r="B30" s="58" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C30" s="71" t="n">
+        <v>10788</v>
+      </c>
+      <c r="D30" s="71" t="n">
+        <v>5567</v>
+      </c>
+      <c r="E30" s="71" t="n">
+        <v>5481</v>
+      </c>
+      <c r="F30" s="60" t="n">
+        <v>21836</v>
+      </c>
+    </row>
+    <row r="31" ht="17.1" customHeight="1" s="32">
+      <c r="A31" s="61" t="inlineStr">
+        <is>
+          <t>26 Sep</t>
+        </is>
+      </c>
+      <c r="B31" s="62" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C31" s="72" t="n">
+        <v>8761</v>
+      </c>
+      <c r="D31" s="72" t="n">
+        <v>6029</v>
+      </c>
+      <c r="E31" s="72" t="n">
+        <v>7264.95</v>
+      </c>
+      <c r="F31" s="60" t="n">
+        <v>22054.95</v>
+      </c>
+    </row>
+    <row r="32" ht="17.1" customHeight="1" s="32">
+      <c r="A32" s="61" t="inlineStr">
+        <is>
+          <t>27 Sep</t>
+        </is>
+      </c>
+      <c r="B32" s="62" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C32" s="72" t="n">
+        <v>13134</v>
+      </c>
+      <c r="D32" s="72" t="n">
+        <v>8005</v>
+      </c>
+      <c r="E32" s="72" t="n">
+        <v>13896.75</v>
+      </c>
+      <c r="F32" s="60" t="n">
+        <v>35035.75</v>
+      </c>
+    </row>
+    <row r="33" ht="17.1" customHeight="1" s="32">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>28 Sep</t>
+        </is>
+      </c>
+      <c r="B33" s="58" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C33" s="71" t="n">
+        <v>9034</v>
+      </c>
+      <c r="D33" s="71" t="n">
+        <v>4999</v>
+      </c>
+      <c r="E33" s="71" t="n">
+        <v>9155.5</v>
+      </c>
+      <c r="F33" s="60" t="n">
+        <v>23188.5</v>
+      </c>
+    </row>
+    <row r="34" ht="17.1" customHeight="1" s="32">
+      <c r="A34" s="57" t="inlineStr">
+        <is>
+          <t>29 Sep</t>
+        </is>
+      </c>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C34" s="71" t="n">
+        <v>6928</v>
+      </c>
+      <c r="D34" s="71" t="n">
+        <v>5337</v>
+      </c>
+      <c r="E34" s="71" t="n">
+        <v>5320.75</v>
+      </c>
+      <c r="F34" s="60" t="n">
+        <v>17585.75</v>
+      </c>
+    </row>
+    <row r="35" ht="17.1" customHeight="1" s="32">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>30 Sep</t>
+        </is>
+      </c>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C35" s="71" t="n">
+        <v>9894</v>
+      </c>
+      <c r="D35" s="71" t="n">
+        <v>5316</v>
+      </c>
+      <c r="E35" s="71" t="n">
+        <v>7333</v>
+      </c>
+      <c r="F35" s="60" t="n">
+        <v>22543</v>
+      </c>
+    </row>
+    <row r="36" ht="21.95" customHeight="1" s="32">
+      <c r="A36" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B36" s="66" t="n"/>
+      <c r="C36" s="67" t="n">
+        <v>109838</v>
+      </c>
+      <c r="D36" s="67" t="n">
+        <v>77089</v>
+      </c>
+      <c r="E36" s="67" t="n">
+        <v>68509.03</v>
+      </c>
+      <c r="F36" s="68" t="n">
+        <v>255436.03</v>
+      </c>
+    </row>
+    <row r="37" ht="21.95" customHeight="1" s="32">
+      <c r="A37" s="69" t="inlineStr">
+        <is>
+          <t>ZONE TOTAL  —  MONTH OF SEPTEMBER 2026</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="n"/>
+      <c r="C37" s="40" t="n"/>
+      <c r="D37" s="40" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="70" t="n">
+        <v>255436.03</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A37:E37"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>